<commit_message>
split flatten logic from to_pandas py
</commit_message>
<xml_diff>
--- a/reconcile/storage/output/reconciliation_outputs_factory.xlsx
+++ b/reconcile/storage/output/reconciliation_outputs_factory.xlsx
@@ -874,7 +874,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1356,7 +1356,7 @@
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -4700,7 +4700,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>['']</t>
+          <t>[nan]</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">

</xml_diff>